<commit_message>
casted down to proper type
</commit_message>
<xml_diff>
--- a/rustysort/test/small_input.xlsx
+++ b/rustysort/test/small_input.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Amrit\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\amrit\Desktop\Callsort\rustysort\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54357730-86C4-4A9C-ACCA-344B360CEF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63300B4D-8185-4D4A-87AD-2404ED24CC9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4665" yWindow="4290" windowWidth="28800" windowHeight="15345" xr2:uid="{EECB155A-459E-1940-B529-75A0F0CD5F8C}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{EECB155A-459E-1940-B529-75A0F0CD5F8C}"/>
   </bookViews>
   <sheets>
     <sheet name="input" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>instance_title</t>
   </si>
@@ -1094,6 +1094,18 @@
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1">
+        <v>31300000000000</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>